<commit_message>
Give every project its own visual identity
Replace the shared green and amber theme with a look designed for each
fictional business, rebuild all covers with varied compositions from
fresh screenshots, restyle the documents and the portfolio home page,
and rebuild the source packages. Existing checks still pass.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WtPVhc7jkXrXagMiRq32Hw
</commit_message>
<xml_diff>
--- a/03-financial-report-Expense_Report_Sample.xlsx
+++ b/03-financial-report-Expense_Report_Sample.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\Codex-Utopia\PROJECTS\competition-operations\WORK\CURRENT\portfolio-quality-20261019\documents\out\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9715AF3-AD78-43BE-BD39-8C0BF796C2B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B81BD00B-F136-4581-9991-570A21A7DE33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="300" yWindow="345" windowWidth="28140" windowHeight="14835" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -378,11 +378,11 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="4">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
-    <numFmt numFmtId="165" formatCode="#,##0.00;\(#,##0.00\);&quot;-&quot;"/>
+    <numFmt numFmtId="165" formatCode="#,##0.00_);\(#,##0.00\);&quot;-&quot;_)"/>
     <numFmt numFmtId="166" formatCode="mmm\ yyyy"/>
-    <numFmt numFmtId="167" formatCode="0.0%;\(0.0%\);&quot;-&quot;"/>
+    <numFmt numFmtId="167" formatCode="0.0%_);\(0.0%\);&quot;-&quot;_)"/>
   </numFmts>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -392,42 +392,46 @@
     </font>
     <font>
       <b/>
-      <sz val="10"/>
-      <color rgb="FF13201B"/>
-      <name val="Arial"/>
+      <sz val="11"/>
+      <color rgb="FF1F2328"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <sz val="10"/>
-      <color rgb="FF0000FF"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color rgb="FF5D6F66"/>
-      <name val="Arial"/>
+      <color rgb="FF5F6368"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <sz val="10"/>
+      <sz val="11"/>
       <color rgb="FFFFFFFF"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
     </font>
     <font>
-      <sz val="10"/>
-      <color rgb="FF13201B"/>
-      <name val="Arial"/>
+      <sz val="11"/>
+      <color rgb="FF1F2328"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="18"/>
+      <color rgb="FF1F2328"/>
+      <name val="Georgia"/>
+    </font>
+    <font>
+      <sz val="13"/>
+      <color rgb="FF1F2328"/>
+      <name val="Georgia"/>
     </font>
     <font>
       <b/>
-      <sz val="16"/>
-      <color rgb="FF13201B"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="12"/>
-      <color rgb="FF13201B"/>
-      <name val="Arial"/>
+      <sz val="11"/>
+      <color rgb="FF7D4E6B"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="4">
@@ -439,12 +443,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF0E3B2B"/>
+        <fgColor rgb="FF2E3238"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFEAF1EC"/>
+        <fgColor rgb="FFF3ECF1"/>
       </patternFill>
     </fill>
   </fills>
@@ -461,7 +465,7 @@
       <right/>
       <top/>
       <bottom style="thin">
-        <color rgb="FFDFE3DC"/>
+        <color rgb="FFDCDDE0"/>
       </bottom>
       <diagonal/>
     </border>
@@ -469,10 +473,10 @@
       <left/>
       <right/>
       <top style="medium">
-        <color rgb="FF13201B"/>
+        <color rgb="FF1F2328"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFDFE3DC"/>
+        <color rgb="FFDCDDE0"/>
       </bottom>
       <diagonal/>
     </border>
@@ -480,10 +484,10 @@
       <left/>
       <right/>
       <top style="medium">
-        <color rgb="FF13201B"/>
+        <color rgb="FF7D4E6B"/>
       </top>
       <bottom style="medium">
-        <color rgb="FF13201B"/>
+        <color rgb="FF7D4E6B"/>
       </bottom>
       <diagonal/>
     </border>
@@ -528,11 +532,11 @@
     <xf numFmtId="166" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="1" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="8" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="167" fontId="1" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="8" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -556,41 +560,47 @@
     <dxf>
       <font>
         <b/>
-        <sz val="10"/>
+        <sz val="11"/>
         <color rgb="FFB4412F"/>
-        <name val="Arial"/>
+        <name val="Calibri"/>
       </font>
     </dxf>
     <dxf>
       <font>
         <b/>
-        <sz val="10"/>
+        <sz val="11"/>
         <color rgb="FFB4412F"/>
-        <name val="Arial"/>
+        <name val="Calibri"/>
       </font>
     </dxf>
     <dxf>
       <font>
         <b/>
-        <sz val="10"/>
+        <sz val="11"/>
         <color rgb="FFB4412F"/>
-        <name val="Arial"/>
+        <name val="Calibri"/>
       </font>
     </dxf>
     <dxf>
       <font>
         <b/>
-        <sz val="10"/>
-        <color rgb="FF175841"/>
-        <name val="Arial"/>
+        <sz val="11"/>
+        <color rgb="FF7D4E6B"/>
+        <name val="Calibri"/>
       </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF3ECF1"/>
+          <bgColor rgb="FFF3ECF1"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
       <font>
         <b/>
-        <sz val="10"/>
+        <sz val="11"/>
         <color rgb="FFB4412F"/>
-        <name val="Arial"/>
+        <name val="Calibri"/>
       </font>
     </dxf>
   </dxfs>
@@ -636,11 +646,11 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="175841"/>
+              <a:srgbClr val="7D4E6B"/>
             </a:solidFill>
             <a:ln>
               <a:solidFill>
-                <a:srgbClr val="175841"/>
+                <a:srgbClr val="7D4E6B"/>
               </a:solidFill>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -677,7 +687,7 @@
             <c:numRef>
               <c:f>Summary!$B$14:$B$19</c:f>
               <c:numCache>
-                <c:formatCode>#,##0.00;\(#,##0.00\);"-"</c:formatCode>
+                <c:formatCode>#,##0.00_);\(#,##0.00\);"-"_)</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
                   <c:v>1678.69</c:v>
@@ -709,7 +719,7 @@
                   </a:solidFill>
                   <a:ln>
                     <a:solidFill>
-                      <a:srgbClr val="175841"/>
+                      <a:srgbClr val="7D4E6B"/>
                     </a:solidFill>
                     <a:prstDash val="solid"/>
                   </a:ln>
@@ -717,7 +727,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-BD46-433C-94EA-C16EEFAB09C4}"/>
+              <c16:uniqueId val="{00000000-93E3-4596-82C9-F3C2551DCA16}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -737,11 +747,11 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="93B3A0"/>
+              <a:srgbClr val="BFC3C8"/>
             </a:solidFill>
             <a:ln>
               <a:solidFill>
-                <a:srgbClr val="93B3A0"/>
+                <a:srgbClr val="BFC3C8"/>
               </a:solidFill>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -778,7 +788,7 @@
             <c:numRef>
               <c:f>Summary!$C$14:$C$19</c:f>
               <c:numCache>
-                <c:formatCode>#,##0.00;\(#,##0.00\);"-"</c:formatCode>
+                <c:formatCode>#,##0.00_);\(#,##0.00\);"-"_)</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
                   <c:v>2100</c:v>
@@ -810,7 +820,7 @@
                   </a:solidFill>
                   <a:ln>
                     <a:solidFill>
-                      <a:srgbClr val="93B3A0"/>
+                      <a:srgbClr val="BFC3C8"/>
                     </a:solidFill>
                     <a:prstDash val="solid"/>
                   </a:ln>
@@ -818,7 +828,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-BD46-433C-94EA-C16EEFAB09C4}"/>
+              <c16:uniqueId val="{00000001-93E3-4596-82C9-F3C2551DCA16}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -863,7 +873,7 @@
           <c:spPr>
             <a:ln>
               <a:solidFill>
-                <a:srgbClr val="DFE3DC"/>
+                <a:srgbClr val="DCDDE0"/>
               </a:solidFill>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1254,7 +1264,7 @@
     <col min="7" max="14" width="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="20.25" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1327,7 +1337,7 @@
         <v>1832.4733333333334</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A12" s="9" t="s">
         <v>9</v>
       </c>
@@ -1504,7 +1514,7 @@
         <v>0.87260634920634916</v>
       </c>
     </row>
-    <row r="22" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A22" s="9" t="s">
         <v>16</v>
       </c>
@@ -1635,7 +1645,7 @@
         <v>0.87260634920634916</v>
       </c>
     </row>
-    <row r="30" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A30" s="9" t="s">
         <v>18</v>
       </c>
@@ -1667,7 +1677,7 @@
         <v>OK</v>
       </c>
     </row>
-    <row r="35" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:2" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A35" s="9" t="s">
         <v>22</v>
       </c>

</xml_diff>